<commit_message>
store-manager: weekly dashboard + report builders to week of 2026-06-28
</commit_message>
<xml_diff>
--- a/Canton_Collective_Weekly_Report.xlsx
+++ b/Canton_Collective_Weekly_Report.xlsx
@@ -92,7 +92,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Canton Collective — Weekly Performance · May 11 – Jun 21, 2026 (GMV = total_sales)</t>
+          <t xml:space="preserve">Canton Collective — Weekly Performance · May 11 – Jun 28, 2026 (GMV = total_sales)</t>
         </is>
       </c>
     </row>
@@ -102,7 +102,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">KPIs — all 6 weeks</t>
+          <t xml:space="preserve">KPIs — all 7 weeks</t>
         </is>
       </c>
     </row>
@@ -423,114 +423,158 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>19353.59</v>
+      </c>
+      <c r="C11">
+        <v>184</v>
+      </c>
+      <c r="D11">
+        <v>101.75</v>
+      </c>
+      <c r="E11">
+        <v>31496</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.51%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+39.1%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+27.8%</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-12.3%</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BETTER</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Key findings</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">#</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Finding</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEADLINE (Jun 15–21): MAMC overtakes 1Jinn Studio as #1 vendor for the first time — 39.0% vs 25.7% (MAMC +16.7pp WoW, 1Jinn −9.8pp).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verdict WORSE: GMV $13,916.50, −7.7% WoW, −11.2% vs trailing 4-wk avg.</t>
+          <t xml:space="preserve">HEADLINE (Jun 22–28): Breakout week — GMV $19,353.59, +39.1% WoW and +27.8% vs 4-wk avg (BETTER), best in trailing-8.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conversion stays soft: CVR 0.56→0.44→0.42% over 3 weeks; browse→cart leak persists. Traffic flat (~26K sessions).</t>
+          <t xml:space="preserve">MAMC pulls away to 44.1% share (+5.1pp) — runaway #1, supplies all top-3 heroes incl. NEW #1 Dreamy Underwater Garden Slip Maxi ($1,528).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AOV slipped off its peak: $108.00 → $106.56 after climbing every week May–early June.</t>
+          <t xml:space="preserve">2th Desire collapses −6.4pp to 6.0% (only Retro Camisole Layer Top holding); Outtheblue recovers 0.8%→3.7% (+2.9pp).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAMC win is broad (12 SKUs selling): Lavender Floral hero $847, NEW climber Dusty Rose Bandeau $737, Green Fold Over Skirt $607.</t>
+          <t xml:space="preserve">Driver: traffic surge (+21%, ~31.5K sessions) AND conversion recovery (+20%, CVR 0.42→0.51%) — the 3-week browse→cart leak eased across the whole funnel.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">1Jinn Studio ceding share 46% → 26% since mid-May; Outtheblue spiked then faded (6.6% → 0.8%).</t>
+          <t xml:space="preserve">Full-funnel recovery: cart-add 3.57→3.76%, reach-checkout 1.06→1.17%, completion 0.42→0.51%.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Email underutilized: 1 send this week (0617 2th Desire) $75 / 1 conv at 61.5% open; 7 campaigns ~$819 attributed total.</t>
+          <t xml:space="preserve">AOV a mild drag: $106.56 → $101.75 as orders jumped +44% (184 orders).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blind spot: Meta CC ad account (SGD) UNSETTLED / not queryable — paid-social spend unverified.</t>
+          <t xml:space="preserve">Email underutilized: 1 send this week (0623 Delete-Ex) $133 / 1 conv at 60.2% open; 8 campaigns ~$952 attributed total (email ≈0.7% of GMV) — and pushing a small vendor, not MAMC.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22">
+        <v>8</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blind spot: Meta CC ad account (SGD) UNSETTLED / not queryable — cannot confirm if the traffic surge was paid-driven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
         <v>9</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YoY −37.2% vs Jun 2025 (214 orders @ $97 last year vs 128 @ $107 now) — June 2025 already scaled.</t>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY −12.3% vs Jun 2025 (195 orders @ ~$111 last year vs 184 @ $102 now) — gap narrowing sharply from −37% last week.</t>
         </is>
       </c>
     </row>
@@ -1575,21 +1619,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lavender Floral Chiffon Slip Mini Dress (MAMC)</t>
+          <t xml:space="preserve">Dreamy Underwater Garden Slip Maxi Dress (MAMC)</t>
         </is>
       </c>
       <c r="B49">
         <v>0</v>
       </c>
       <c r="C49">
-        <v>512.05</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>1201.2</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLIMBER / hero</t>
+          <t xml:space="preserve">NEW #1 hero</t>
         </is>
       </c>
     </row>
@@ -1610,140 +1654,140 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEW CLIMBER</t>
+          <t xml:space="preserve">CLIMBER → hero (broad)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Fold Over Asymmetric Hem Midi Skirt (MAMC)</t>
+          <t xml:space="preserve">Lavender Floral Chiffon Slip Mini Dress (MAMC)</t>
         </is>
       </c>
       <c r="B51">
         <v>0</v>
       </c>
       <c r="C51">
-        <v>0</v>
+        <v>512.05</v>
       </c>
       <c r="D51">
-        <v>391</v>
+        <v>1201.2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLIMBER</t>
+          <t xml:space="preserve">Hero (holding)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ruffle Trim Gingham Babydoll Mini Dress (MAMC)</t>
+          <t xml:space="preserve">Polka Dot Stripe Henley Tank 3pc Set (1Jinn)</t>
         </is>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>761.92</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>507.99</v>
       </c>
       <c r="D52">
-        <v>295.63</v>
+        <v>464.84</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emerging</t>
+          <t xml:space="preserve">Rebounded</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retro Camisole Layer Top (2th Desire)</t>
+          <t xml:space="preserve">Y2K Beaded Multi Strap Top (1Jinn)</t>
         </is>
       </c>
       <c r="B53">
-        <v>803.61</v>
+        <v>522.69</v>
       </c>
       <c r="C53">
-        <v>344.34</v>
+        <v>616.46</v>
       </c>
       <c r="D53">
-        <v>276.58</v>
+        <v>321.2</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Volatile core</t>
+          <t xml:space="preserve">Core, oscillating</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y2K Beaded Multi Strap Top</t>
+          <t xml:space="preserve">Shell Buttons Front Puff Sleeve Shirt (Deleteex)</t>
         </is>
       </c>
       <c r="B54">
-        <v>522.69</v>
+        <v>705.29</v>
       </c>
       <c r="C54">
-        <v>616.46</v>
+        <v>567.11</v>
       </c>
       <c r="D54">
-        <v>321.2</v>
+        <v>361.65</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Core, oscillating</t>
+          <t xml:space="preserve">Soft core</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shell Buttons Front Puff Sleeve Shirt</t>
+          <t xml:space="preserve">Retro Camisole Layer Top (2th Desire)</t>
         </is>
       </c>
       <c r="B55">
-        <v>705.29</v>
+        <v>803.61</v>
       </c>
       <c r="C55">
-        <v>567.11</v>
+        <v>344.34</v>
       </c>
       <c r="D55">
-        <v>361.65</v>
+        <v>276.58</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Soft core</t>
+          <t xml:space="preserve">2TH lone holdout</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midnight Meow Zip Up Cat Ear Hoodie</t>
+          <t xml:space="preserve">Green Fold Over Asymmetric Hem Midi Skirt (MAMC)</t>
         </is>
       </c>
       <c r="B56">
-        <v>422.96</v>
+        <v>0</v>
       </c>
       <c r="C56">
-        <v>569.26</v>
+        <v>0</v>
       </c>
       <c r="D56">
-        <v>580.26</v>
+        <v>391</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fading</t>
+          <t xml:space="preserve">Cooling</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metal Flower Pleated Strapless Mini Dress</t>
+          <t xml:space="preserve">Metal Flower Pleated Strapless Mini Dress (1Jinn)</t>
         </is>
       </c>
       <c r="B57">
@@ -1757,168 +1801,210 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECLINING (gone)</t>
+          <t xml:space="preserve">Rebounded</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polka Dot Stripe Henley Tank 3pc Set</t>
+          <t xml:space="preserve">Midnight Meow Zip Up Cat Ear Hoodie (1Jinn)</t>
         </is>
       </c>
       <c r="B58">
-        <v>761.92</v>
+        <v>422.96</v>
       </c>
       <c r="C58">
-        <v>507.99</v>
+        <v>569.26</v>
       </c>
       <c r="D58">
-        <v>464.84</v>
+        <v>580.26</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECLINING (gone)</t>
+          <t xml:space="preserve">Fading</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59"/>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ruffle Trim Gingham Babydoll Mini Dress (MAMC)</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>295.63</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiet this wk</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outtheblue line (vendor total)</t>
+        </is>
+      </c>
+      <c r="B60">
+        <v>0</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recovered (+2.9pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Email campaigns (Klaviyo)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Send Date</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Campaign</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Theme</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Recipients</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Open Rate</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Attributed Rev</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Conv</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">May 13</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0513 CC new drop</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New drop</t>
-        </is>
-      </c>
-      <c r="D62">
-        <v>91</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39.6%</t>
-        </is>
-      </c>
-      <c r="F62">
-        <v>71</v>
-      </c>
-      <c r="G62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">May 20</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0520 MAMC</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAMC</t>
-        </is>
-      </c>
-      <c r="D63">
-        <v>457</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32.9%</t>
-        </is>
-      </c>
-      <c r="F63">
-        <v>0</v>
-      </c>
-      <c r="G63">
-        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t xml:space="preserve">May 13</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0513 CC new drop</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New drop</t>
+        </is>
+      </c>
+      <c r="D64">
+        <v>91</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39.6%</t>
+        </is>
+      </c>
+      <c r="F64">
+        <v>71</v>
+      </c>
+      <c r="G64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May 20</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0520 MAMC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MAMC</t>
+        </is>
+      </c>
+      <c r="D65">
+        <v>457</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32.9%</t>
+        </is>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t xml:space="preserve">May 27</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t xml:space="preserve">0527 MAMC</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t xml:space="preserve">MAMC</t>
         </is>
       </c>
-      <c r="D64">
+      <c r="D66">
         <v>774</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t xml:space="preserve">34.4%</t>
         </is>
       </c>
-      <c r="F64">
+      <c r="F66">
         <v>41</v>
       </c>
-      <c r="G64">
+      <c r="G66">
         <v>1</v>
       </c>
     </row>
@@ -1937,6 +2023,7 @@
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2131,1210 +2218,1534 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>19353.59</v>
+      </c>
+      <c r="C6">
+        <v>184</v>
+      </c>
+      <c r="D6">
+        <v>101.75</v>
+      </c>
+      <c r="E6">
+        <v>31496</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.51%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+39.1%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+27.8%</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-12.3%</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BETTER</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">WHY — decomposition (GMV = Sessions × Conv Rate × AOV)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Transition</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Sessions Δ</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Conv Rate Δ</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">AOV Δ</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Orders Δ</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">GMV Δ</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Primary driver</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">May 25 → Jun 01</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+6.6%</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+17.2%</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+5.9%</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+16.4%</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+27.0%</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Broad-based: all three positive</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jun 01 → Jun 08</t>
+          <t xml:space="preserve">May 25 → Jun 01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-3.8%</t>
+          <t xml:space="preserve">+6.6%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-21.7%</t>
+          <t xml:space="preserve">+17.2%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">+2.2%</t>
+          <t xml:space="preserve">+5.9%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-18.4%</t>
+          <t xml:space="preserve">+16.4%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-14.7%</t>
+          <t xml:space="preserve">+27.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONVERSION collapse (browse→cart)</t>
+          <t xml:space="preserve">Broad-based: all three positive</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t xml:space="preserve">Jun 01 → Jun 08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-3.8%</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-21.7%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+2.2%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-18.4%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-14.7%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONVERSION collapse (browse→cart)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Jun 08 → Jun 15</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve">+0.2%</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t xml:space="preserve">-2.9%</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t xml:space="preserve">-1.3%</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">-3.8%</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t xml:space="preserve">-7.7%</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t xml:space="preserve">Conversion stays soft + AOV slips off peak (traffic flat)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 15 → Jun 22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+21.5%</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+19.8%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-4.5%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+43.8%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+39.1%</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traffic surge + CONVERSION recovery (browse→cart leak eases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Funnel + discounts &amp; returns</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Week</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Sessions</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Cart Adds</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Reached Checkout</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Completed</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Conv Rate</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Discounts</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Returns</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 1–7</t>
-        </is>
-      </c>
-      <c r="B15">
-        <v>26887</v>
-      </c>
-      <c r="C15">
-        <v>1042</v>
-      </c>
-      <c r="D15">
-        <v>327</v>
-      </c>
-      <c r="E15">
-        <v>150</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.56%</t>
-        </is>
-      </c>
-      <c r="G15">
-        <v>-1822.65</v>
-      </c>
-      <c r="H15">
-        <v>-1016.1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 8–14</t>
-        </is>
-      </c>
-      <c r="B16">
-        <v>25874</v>
-      </c>
-      <c r="C16">
-        <v>869</v>
-      </c>
-      <c r="D16">
-        <v>289</v>
-      </c>
-      <c r="E16">
-        <v>113</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.44%</t>
-        </is>
-      </c>
-      <c r="G16">
-        <v>-2177.46</v>
-      </c>
-      <c r="H16">
-        <v>-428.99</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t xml:space="preserve">Jun 1–7</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>26887</v>
+      </c>
+      <c r="C17">
+        <v>1042</v>
+      </c>
+      <c r="D17">
+        <v>327</v>
+      </c>
+      <c r="E17">
+        <v>150</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.56%</t>
+        </is>
+      </c>
+      <c r="G17">
+        <v>-1822.65</v>
+      </c>
+      <c r="H17">
+        <v>-1016.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 8–14</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>25874</v>
+      </c>
+      <c r="C18">
+        <v>869</v>
+      </c>
+      <c r="D18">
+        <v>289</v>
+      </c>
+      <c r="E18">
+        <v>113</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.44%</t>
+        </is>
+      </c>
+      <c r="G18">
+        <v>-2177.46</v>
+      </c>
+      <c r="H18">
+        <v>-428.99</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t xml:space="preserve">Jun 15–21</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B19">
         <v>25933</v>
       </c>
-      <c r="C17">
+      <c r="C19">
         <v>925</v>
       </c>
-      <c r="D17">
+      <c r="D19">
         <v>275</v>
       </c>
-      <c r="E17">
+      <c r="E19">
         <v>110</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">0.42%</t>
         </is>
       </c>
-      <c r="G17">
+      <c r="G19">
         <v>-1498.37</v>
       </c>
-      <c r="H17">
+      <c r="H19">
         <v>-561.62</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>31496</v>
+      </c>
+      <c r="C20">
+        <v>1184</v>
+      </c>
+      <c r="D20">
+        <v>367</v>
+      </c>
+      <c r="E20">
+        <v>160</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.51%</t>
+        </is>
+      </c>
+      <c r="G20">
+        <v>-2645.97</v>
+      </c>
+      <c r="H20">
+        <v>-625.34</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Traffic by referrer source</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Week</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Direct/Unknown $</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ord</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Social $</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ord</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Search $</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ord</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t xml:space="preserve">Jun 1–7</t>
         </is>
       </c>
-      <c r="B21">
+      <c r="B24">
         <v>11588.8</v>
       </c>
-      <c r="C21">
+      <c r="C24">
         <v>104</v>
       </c>
-      <c r="D21">
+      <c r="D24">
         <v>3483.83</v>
       </c>
-      <c r="E21">
+      <c r="E24">
         <v>33</v>
       </c>
-      <c r="F21">
+      <c r="F24">
         <v>2591.33</v>
       </c>
-      <c r="G21">
+      <c r="G24">
         <v>26</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t xml:space="preserve">Jun 8–14</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B25">
         <v>9522.26</v>
       </c>
-      <c r="C22">
+      <c r="C25">
         <v>82</v>
       </c>
-      <c r="D22">
+      <c r="D25">
         <v>3767.02</v>
       </c>
-      <c r="E22">
+      <c r="E25">
         <v>35</v>
       </c>
-      <c r="F22">
+      <c r="F25">
         <v>1785.6</v>
       </c>
-      <c r="G22">
+      <c r="G25">
         <v>16</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">Jun 15–21</t>
         </is>
       </c>
-      <c r="B23">
+      <c r="B26">
         <v>9299.36</v>
       </c>
-      <c r="C23">
+      <c r="C26">
         <v>78</v>
       </c>
-      <c r="D23">
+      <c r="D26">
         <v>2901.45</v>
       </c>
-      <c r="E23">
+      <c r="E26">
         <v>33</v>
       </c>
-      <c r="F23">
+      <c r="F26">
         <v>1715.69</v>
       </c>
-      <c r="G23">
+      <c r="G26">
         <v>17</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vendor GMV share (% of store)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vendor</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 1–7</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 8–14</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 15–21</t>
-        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">1Jinn Studio</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31.4%</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">35.5%</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">25.7%</t>
-        </is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="B27">
+        <v>11873.51</v>
+      </c>
+      <c r="C27">
+        <v>109</v>
+      </c>
+      <c r="D27">
+        <v>4334.89</v>
+      </c>
+      <c r="E27">
+        <v>45</v>
+      </c>
+      <c r="F27">
+        <v>3145.19</v>
+      </c>
+      <c r="G27">
+        <v>30</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAMC</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21.5%</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22.3%</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39.0%</t>
-        </is>
-      </c>
+      <c r="A28"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2th Desire</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20.6%</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13.2%</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12.4%</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vendor GMV share (% of store)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deleteex</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12.5%</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13.8%</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11.4%</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vendor</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 1–7</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 8–14</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 15–21</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">First Floor</t>
+          <t xml:space="preserve">1Jinn Studio</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6%</t>
+          <t xml:space="preserve">31.4%</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.1%</t>
+          <t xml:space="preserve">35.5%</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.0%</t>
+          <t xml:space="preserve">25.7%</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24.7%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outtheblue</t>
+          <t xml:space="preserve">MAMC</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4%</t>
+          <t xml:space="preserve">21.5%</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.6%</t>
+          <t xml:space="preserve">22.3%</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.8%</t>
+          <t xml:space="preserve">39.0%</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44.1%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">1Jinn M2M</t>
+          <t xml:space="preserve">2th Desire</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4%</t>
+          <t xml:space="preserve">20.6%</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.4%</t>
+          <t xml:space="preserve">13.2%</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4%</t>
+          <t xml:space="preserve">12.4%</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.0%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">(blank = shipping)</t>
+          <t xml:space="preserve">Deleteex</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.1%</t>
+          <t xml:space="preserve">12.5%</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.9%</t>
+          <t xml:space="preserve">13.8%</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.2%</t>
+          <t xml:space="preserve">11.4%</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11.5%</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First Floor</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.6%</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.1%</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.0%</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.7%</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vendor GMV ($)</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outtheblue</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4%</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.6%</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.8%</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.7%</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vendor</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 1–7</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 8–14</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 15–21</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1Jinn M2M</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4%</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.4%</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4%</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.0%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">1Jinn Studio</t>
-        </is>
-      </c>
-      <c r="B38">
-        <v>5554.53</v>
-      </c>
-      <c r="C38">
-        <v>5355.42</v>
-      </c>
-      <c r="D38">
-        <v>3572.62</v>
+          <t xml:space="preserve">(blank = shipping)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7.1%</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.9%</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.2%</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.3%</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAMC</t>
-        </is>
-      </c>
-      <c r="B39">
-        <v>3805.37</v>
-      </c>
-      <c r="C39">
-        <v>3354.41</v>
-      </c>
-      <c r="D39">
-        <v>5424.71</v>
-      </c>
+      <c r="A39"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2th Desire</t>
-        </is>
-      </c>
-      <c r="B40">
-        <v>3642.84</v>
-      </c>
-      <c r="C40">
-        <v>1985.62</v>
-      </c>
-      <c r="D40">
-        <v>1725.62</v>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vendor GMV ($)</t>
+        </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deleteex</t>
-        </is>
-      </c>
-      <c r="B41">
-        <v>2211.05</v>
-      </c>
-      <c r="C41">
-        <v>2078.62</v>
-      </c>
-      <c r="D41">
-        <v>1590.93</v>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vendor</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 1–7</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 8–14</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 15–21</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">First Floor</t>
+          <t xml:space="preserve">1Jinn Studio</t>
         </is>
       </c>
       <c r="B42">
-        <v>804.64</v>
+        <v>5554.53</v>
       </c>
       <c r="C42">
-        <v>459.99</v>
+        <v>5355.42</v>
       </c>
       <c r="D42">
-        <v>555.49</v>
+        <v>3572.62</v>
+      </c>
+      <c r="E42">
+        <v>4778.88</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outtheblue</t>
+          <t xml:space="preserve">MAMC</t>
         </is>
       </c>
       <c r="B43">
-        <v>79</v>
+        <v>3805.37</v>
       </c>
       <c r="C43">
-        <v>989.58</v>
+        <v>3354.41</v>
       </c>
       <c r="D43">
-        <v>109.97</v>
+        <v>5424.71</v>
+      </c>
+      <c r="E43">
+        <v>8536.78</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">1Jinn M2M</t>
+          <t xml:space="preserve">2th Desire</t>
         </is>
       </c>
       <c r="B44">
-        <v>241.03</v>
+        <v>3642.84</v>
       </c>
       <c r="C44">
-        <v>55.16</v>
+        <v>1985.62</v>
       </c>
       <c r="D44">
-        <v>198.03</v>
+        <v>1725.62</v>
+      </c>
+      <c r="E44">
+        <v>1170.45</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">(blank = shipping)</t>
+          <t xml:space="preserve">Deleteex</t>
         </is>
       </c>
       <c r="B45">
-        <v>1254.6</v>
+        <v>2211.05</v>
       </c>
       <c r="C45">
-        <v>740.08</v>
+        <v>2078.62</v>
       </c>
       <c r="D45">
-        <v>725.2</v>
+        <v>1590.93</v>
+      </c>
+      <c r="E45">
+        <v>2223.69</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First Floor</t>
+        </is>
+      </c>
+      <c r="B46">
+        <v>804.64</v>
+      </c>
+      <c r="C46">
+        <v>459.99</v>
+      </c>
+      <c r="D46">
+        <v>555.49</v>
+      </c>
+      <c r="E46">
+        <v>715.57</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Top products — GMV by week</t>
-        </is>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outtheblue</t>
+        </is>
+      </c>
+      <c r="B47">
+        <v>79</v>
+      </c>
+      <c r="C47">
+        <v>989.58</v>
+      </c>
+      <c r="D47">
+        <v>109.97</v>
+      </c>
+      <c r="E47">
+        <v>712.64</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 1–7</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 8–14</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun 15–21</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trend</t>
-        </is>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1Jinn M2M</t>
+        </is>
+      </c>
+      <c r="B48">
+        <v>241.03</v>
+      </c>
+      <c r="C48">
+        <v>55.16</v>
+      </c>
+      <c r="D48">
+        <v>198.03</v>
+      </c>
+      <c r="E48">
+        <v>196.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lavender Floral Chiffon Slip Mini Dress (MAMC)</t>
+          <t xml:space="preserve">(blank = shipping)</t>
         </is>
       </c>
       <c r="B49">
-        <v>1197.35</v>
+        <v>1254.6</v>
       </c>
       <c r="C49">
-        <v>771.16</v>
+        <v>740.08</v>
       </c>
       <c r="D49">
-        <v>847.43</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLIMBER / hero</t>
-        </is>
+        <v>725.2</v>
+      </c>
+      <c r="E49">
+        <v>1018.98</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dusty Rose Layered Gauze Bandeau Top (MAMC)</t>
-        </is>
-      </c>
-      <c r="B50">
-        <v>0</v>
-      </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-      <c r="D50">
-        <v>737.11</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEW CLIMBER</t>
-        </is>
-      </c>
+      <c r="A50"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Green Fold Over Asymmetric Hem Midi Skirt (MAMC)</t>
-        </is>
-      </c>
-      <c r="B51">
-        <v>326.4</v>
-      </c>
-      <c r="C51">
-        <v>397.63</v>
-      </c>
-      <c r="D51">
-        <v>607.41</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLIMBER</t>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Top products — GMV by week</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ruffle Trim Gingham Babydoll Mini Dress (MAMC)</t>
-        </is>
-      </c>
-      <c r="B52">
-        <v>0</v>
-      </c>
-      <c r="C52">
-        <v>432.67</v>
-      </c>
-      <c r="D52">
-        <v>159.8</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emerging</t>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 1–7</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 8–14</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 15–21</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trend</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retro Camisole Layer Top (2th Desire)</t>
+          <t xml:space="preserve">Dreamy Underwater Garden Slip Maxi Dress (MAMC)</t>
         </is>
       </c>
       <c r="B53">
-        <v>693.66</v>
+        <v>0</v>
       </c>
       <c r="C53">
-        <v>547.9</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>397.29</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Volatile core</t>
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>1527.75</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEW #1 hero</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y2K Beaded Multi Strap Top</t>
+          <t xml:space="preserve">Dusty Rose Layered Gauze Bandeau Top (MAMC)</t>
         </is>
       </c>
       <c r="B54">
-        <v>331.17</v>
+        <v>0</v>
       </c>
       <c r="C54">
-        <v>594.51</v>
+        <v>0</v>
       </c>
       <c r="D54">
-        <v>460.85</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Core, oscillating</t>
+        <v>737.11</v>
+      </c>
+      <c r="E54">
+        <v>1471.06</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLIMBER → hero (broad)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shell Buttons Front Puff Sleeve Shirt</t>
+          <t xml:space="preserve">Lavender Floral Chiffon Slip Mini Dress (MAMC)</t>
         </is>
       </c>
       <c r="B55">
-        <v>0</v>
+        <v>1197.35</v>
       </c>
       <c r="C55">
-        <v>458.22</v>
+        <v>771.16</v>
       </c>
       <c r="D55">
-        <v>281.07</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Soft core</t>
+        <v>847.43</v>
+      </c>
+      <c r="E55">
+        <v>987.3</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hero (holding)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midnight Meow Zip Up Cat Ear Hoodie</t>
+          <t xml:space="preserve">Polka Dot Stripe Henley Tank 3pc Set (1Jinn)</t>
         </is>
       </c>
       <c r="B56">
-        <v>530.75</v>
+        <v>464.84</v>
       </c>
       <c r="C56">
-        <v>431.75</v>
+        <v>339.01</v>
       </c>
       <c r="D56">
-        <v>156.74</v>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fading</t>
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>511.33</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rebounded</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metal Flower Pleated Strapless Mini Dress</t>
+          <t xml:space="preserve">Y2K Beaded Multi Strap Top (1Jinn)</t>
         </is>
       </c>
       <c r="B57">
-        <v>0</v>
+        <v>331.17</v>
       </c>
       <c r="C57">
-        <v>0</v>
+        <v>594.51</v>
       </c>
       <c r="D57">
-        <v>0</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECLINING (gone)</t>
+        <v>460.85</v>
+      </c>
+      <c r="E57">
+        <v>498.76</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Core, oscillating</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polka Dot Stripe Henley Tank 3pc Set</t>
+          <t xml:space="preserve">Shell Buttons Front Puff Sleeve Shirt (Deleteex)</t>
         </is>
       </c>
       <c r="B58">
-        <v>464.84</v>
+        <v>0</v>
       </c>
       <c r="C58">
-        <v>339.01</v>
+        <v>458.22</v>
       </c>
       <c r="D58">
+        <v>281.07</v>
+      </c>
+      <c r="E58">
+        <v>396.59</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soft core</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retro Camisole Layer Top (2th Desire)</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>693.66</v>
+      </c>
+      <c r="C59">
+        <v>547.9</v>
+      </c>
+      <c r="D59">
+        <v>397.29</v>
+      </c>
+      <c r="E59">
+        <v>366.3</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2TH lone holdout</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Green Fold Over Asymmetric Hem Midi Skirt (MAMC)</t>
+        </is>
+      </c>
+      <c r="B60">
+        <v>326.4</v>
+      </c>
+      <c r="C60">
+        <v>397.63</v>
+      </c>
+      <c r="D60">
+        <v>607.41</v>
+      </c>
+      <c r="E60">
+        <v>291.22</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cooling</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metal Flower Pleated Strapless Mini Dress (1Jinn)</t>
+        </is>
+      </c>
+      <c r="B61">
         <v>0</v>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECLINING (gone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Email campaigns (Klaviyo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Send Date</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Campaign</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Theme</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recipients</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open Rate</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Attributed Rev</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conv</t>
+      <c r="C61">
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>278.49</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rebounded</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jun 03</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0603 Outthe Blue</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outtheblue</t>
-        </is>
+          <t xml:space="preserve">Midnight Meow Zip Up Cat Ear Hoodie (1Jinn)</t>
+        </is>
+      </c>
+      <c r="B62">
+        <v>530.75</v>
+      </c>
+      <c r="C62">
+        <v>431.75</v>
       </c>
       <c r="D62">
-        <v>428</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">66.0%</t>
-        </is>
-      </c>
-      <c r="F62">
-        <v>56.91</v>
-      </c>
-      <c r="G62">
-        <v>1</v>
+        <v>156.74</v>
+      </c>
+      <c r="E62">
+        <v>225.5</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fading</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jun 10</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0610 Outthe Blue vol.2</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outtheblue</t>
-        </is>
+          <t xml:space="preserve">Ruffle Trim Gingham Babydoll Mini Dress (MAMC)</t>
+        </is>
+      </c>
+      <c r="B63">
+        <v>0</v>
+      </c>
+      <c r="C63">
+        <v>432.67</v>
       </c>
       <c r="D63">
-        <v>536</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">62.1%</t>
-        </is>
-      </c>
-      <c r="F63">
-        <v>258.22</v>
-      </c>
-      <c r="G63">
-        <v>1</v>
+        <v>159.8</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiet this wk</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t xml:space="preserve">Outtheblue line (vendor total)</t>
+        </is>
+      </c>
+      <c r="B64">
+        <v>79</v>
+      </c>
+      <c r="C64">
+        <v>989.58</v>
+      </c>
+      <c r="D64">
+        <v>109.97</v>
+      </c>
+      <c r="E64">
+        <v>712.64</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recovered (+2.9pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email campaigns (Klaviyo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Send Date</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Campaign</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Theme</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recipients</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open Rate</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Attributed Rev</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conv</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 03</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0603 Outthe Blue</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outtheblue</t>
+        </is>
+      </c>
+      <c r="D68">
+        <v>428</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">66.0%</t>
+        </is>
+      </c>
+      <c r="F68">
+        <v>56.91</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 10</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0610 Outthe Blue vol.2</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outtheblue</t>
+        </is>
+      </c>
+      <c r="D69">
+        <v>536</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62.1%</t>
+        </is>
+      </c>
+      <c r="F69">
+        <v>258.22</v>
+      </c>
+      <c r="G69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
           <t xml:space="preserve">Jun 13</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t xml:space="preserve">0613 MAMC</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t xml:space="preserve">MAMC</t>
         </is>
       </c>
-      <c r="D64">
+      <c r="D70">
         <v>536</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t xml:space="preserve">59.6%</t>
         </is>
       </c>
-      <c r="F64">
+      <c r="F70">
         <v>316.7</v>
       </c>
-      <c r="G64">
+      <c r="G70">
         <v>1</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t xml:space="preserve">Jun 17</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t xml:space="preserve">0617 2th Desire</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t xml:space="preserve">2th Desire</t>
         </is>
       </c>
-      <c r="D65">
+      <c r="D71">
         <v>552</v>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t xml:space="preserve">61.5%</t>
         </is>
       </c>
-      <c r="F65">
+      <c r="F71">
         <v>75</v>
       </c>
-      <c r="G65">
+      <c r="G71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 23</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0623 Delete-Ex</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete-Ex</t>
+        </is>
+      </c>
+      <c r="D72">
+        <v>626</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60.2%</t>
+        </is>
+      </c>
+      <c r="F72">
+        <v>133</v>
+      </c>
+      <c r="G72">
         <v>1</v>
       </c>
     </row>
@@ -3549,6 +3960,32 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 22–28</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>19353.59</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wk of Jun 23 2025</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>22070.41</v>
+      </c>
+      <c r="E9">
+        <v>195</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-12.3%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>